<commit_message>
Map: WP-B1 Arthas Moloch — Chart-Welt „Moloch“ an arthas_moloch gelinkt + Opt-in-Name-Override im Welten-Sheet (Session 254)
- map-worlds-core: Welten-Sheet-Spalte Name-Override (display-only; Welt-ID, Matching und Kurations-Ziele bleiben auf dem Excel-Namen), locationId-Override tri-state (leer = nicht angefasst), Legacy-3-Spalten-Header wird weiter gelesen
- import-map-worlds: --sync-curation schreibt das 4-Spalten-Layout; Name-only-Zeilen behalten leere locationId-Zelle
- Kurations-Excel: arthas_moloch → link/moloch (Kuration) + moloch → „Arthas Moloch“ (Welten); per Freigabe eingetragen, via --sync-curation normalisiert
- map-worlds.json/review regeneriert: moloch = Arthas Moloch mit 2 Werken; Abdeckung 1354/1710 (79.2 %), Worklist 237
- test-map-worlds: 47/47 grün (neue Override-Fälle inkl. WP-B1-Szenario); Fahrplan-Haken ✔ 254 + Impl-Report
</commit_message>
<xml_diff>
--- a/scripts/seed-data/source/map-worlds-curation.xlsx
+++ b/scripts/seed-data/source/map-worlds-curation.xlsx
@@ -1355,6 +1355,9 @@
     <t>Arthas Moloch</t>
   </si>
   <si>
+    <t>moloch</t>
+  </si>
+  <si>
     <t>arx_tyrannus</t>
   </si>
   <si>
@@ -2715,6 +2718,12 @@
   </si>
   <si>
     <t>locationId-Override</t>
+  </si>
+  <si>
+    <t>Name-Override</t>
+  </si>
+  <si>
+    <t>WP-B1: Chart-Welt „Moloch“ = Arthas Moloch (nicht Moloch III / Molech)</t>
   </si>
 </sst>
 </file>
@@ -2852,7 +2861,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>19</v>
@@ -6272,15 +6281,21 @@
         <v>1</v>
       </c>
       <c r="D162">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E162" t="s">
+        <v>57</v>
+      </c>
+      <c r="F162" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B163" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C163">
         <v>1</v>
@@ -6292,18 +6307,18 @@
         <v>19</v>
       </c>
       <c r="F163" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K163" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B164" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C164">
         <v>1</v>
@@ -6314,10 +6329,10 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B165" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C165">
         <v>1</v>
@@ -6328,10 +6343,10 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B166" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C166">
         <v>1</v>
@@ -6342,10 +6357,10 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B167" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C167">
         <v>1</v>
@@ -6356,10 +6371,10 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B168" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C168">
         <v>1</v>
@@ -6370,10 +6385,10 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B169" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C169">
         <v>1</v>
@@ -6384,10 +6399,10 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B170" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C170">
         <v>1</v>
@@ -6398,10 +6413,10 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B171" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C171">
         <v>1</v>
@@ -6412,10 +6427,10 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B172" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C172">
         <v>1</v>
@@ -6426,24 +6441,24 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B173" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C173">
         <v>1</v>
       </c>
       <c r="D173">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B174" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C174">
         <v>1</v>
@@ -6467,15 +6482,15 @@
         <v>29</v>
       </c>
       <c r="K174" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B175" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C175">
         <v>1</v>
@@ -6499,15 +6514,15 @@
         <v>15</v>
       </c>
       <c r="K175" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B176" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C176">
         <v>1</v>
@@ -6518,10 +6533,10 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B177" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -6530,15 +6545,15 @@
         <v>0</v>
       </c>
       <c r="K177" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B178" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C178">
         <v>1</v>
@@ -6549,10 +6564,10 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B179" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -6563,10 +6578,10 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B180" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C180">
         <v>1</v>
@@ -6577,10 +6592,10 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B181" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C181">
         <v>1</v>
@@ -6591,10 +6606,10 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B182" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C182">
         <v>1</v>
@@ -6605,10 +6620,10 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B183" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C183">
         <v>1</v>
@@ -6620,18 +6635,18 @@
         <v>19</v>
       </c>
       <c r="F183" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K183" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B184" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C184">
         <v>1</v>
@@ -6642,10 +6657,10 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B185" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C185">
         <v>1</v>
@@ -6656,10 +6671,10 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B186" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C186">
         <v>1</v>
@@ -6670,10 +6685,10 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B187" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C187">
         <v>1</v>
@@ -6684,10 +6699,10 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B188" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C188">
         <v>1</v>
@@ -6711,15 +6726,15 @@
         <v>15</v>
       </c>
       <c r="K188" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B189" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C189">
         <v>1</v>
@@ -6730,10 +6745,10 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B190" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C190">
         <v>1</v>
@@ -6744,10 +6759,10 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B191" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C191">
         <v>1</v>
@@ -6762,15 +6777,15 @@
         <v>24</v>
       </c>
       <c r="K191" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B192" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C192">
         <v>1</v>
@@ -6781,10 +6796,10 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B193" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C193">
         <v>1</v>
@@ -6795,10 +6810,10 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B194" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C194">
         <v>1</v>
@@ -6809,10 +6824,10 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B195" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C195">
         <v>1</v>
@@ -6823,10 +6838,10 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B196" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C196">
         <v>1</v>
@@ -6837,10 +6852,10 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B197" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C197">
         <v>1</v>
@@ -6851,10 +6866,10 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B198" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C198">
         <v>1</v>
@@ -6865,10 +6880,10 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B199" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C199">
         <v>1</v>
@@ -6879,10 +6894,10 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B200" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C200">
         <v>1</v>
@@ -6893,10 +6908,10 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B201" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C201">
         <v>1</v>
@@ -6907,10 +6922,10 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B202" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C202">
         <v>1</v>
@@ -6921,10 +6936,10 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B203" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C203">
         <v>1</v>
@@ -6948,15 +6963,15 @@
         <v>15</v>
       </c>
       <c r="K203" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B204" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C204">
         <v>1</v>
@@ -6967,10 +6982,10 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B205" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C205">
         <v>1</v>
@@ -6994,15 +7009,15 @@
         <v>15</v>
       </c>
       <c r="K205" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B206" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C206">
         <v>1</v>
@@ -7026,15 +7041,15 @@
         <v>29</v>
       </c>
       <c r="K206" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B207" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C207">
         <v>1</v>
@@ -7045,10 +7060,10 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B208" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C208">
         <v>1</v>
@@ -7057,15 +7072,15 @@
         <v>0</v>
       </c>
       <c r="K208" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B209" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C209">
         <v>1</v>
@@ -7080,15 +7095,15 @@
         <v>24</v>
       </c>
       <c r="K209" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B210" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C210">
         <v>1</v>
@@ -7099,10 +7114,10 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B211" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C211">
         <v>1</v>
@@ -7113,10 +7128,10 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B212" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C212">
         <v>1</v>
@@ -7131,15 +7146,15 @@
         <v>33</v>
       </c>
       <c r="K212" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B213" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C213">
         <v>1</v>
@@ -7150,10 +7165,10 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B214" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C214">
         <v>1</v>
@@ -7164,10 +7179,10 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B215" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C215">
         <v>1</v>
@@ -7178,10 +7193,10 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B216" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C216">
         <v>1</v>
@@ -7192,10 +7207,10 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B217" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C217">
         <v>1</v>
@@ -7206,10 +7221,10 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B218" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C218">
         <v>1</v>
@@ -7220,24 +7235,24 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B219" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C219">
         <v>1</v>
       </c>
       <c r="D219">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B220" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C220">
         <v>1</v>
@@ -7248,10 +7263,10 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B221" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C221">
         <v>1</v>
@@ -7262,10 +7277,10 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B222" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C222">
         <v>1</v>
@@ -7276,10 +7291,10 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B223" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C223">
         <v>1</v>
@@ -7290,10 +7305,10 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B224" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C224">
         <v>1</v>
@@ -7304,10 +7319,10 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B225" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C225">
         <v>1</v>
@@ -7318,10 +7333,10 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B226" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C226">
         <v>1</v>
@@ -7345,15 +7360,15 @@
         <v>15</v>
       </c>
       <c r="K226" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B227" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C227">
         <v>1</v>
@@ -7368,15 +7383,15 @@
         <v>24</v>
       </c>
       <c r="K227" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B228" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C228">
         <v>1</v>
@@ -7387,10 +7402,10 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B229" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C229">
         <v>1</v>
@@ -7414,15 +7429,15 @@
         <v>15</v>
       </c>
       <c r="K229" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B230" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C230">
         <v>1</v>
@@ -7433,10 +7448,10 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B231" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C231">
         <v>1</v>
@@ -7456,16 +7471,16 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B232" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C232">
         <v>1</v>
       </c>
       <c r="D232">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E232" t="s">
         <v>13</v>
@@ -7483,15 +7498,15 @@
         <v>29</v>
       </c>
       <c r="K232" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B233" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C233">
         <v>1</v>
@@ -7502,10 +7517,10 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B234" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C234">
         <v>1</v>
@@ -7516,10 +7531,10 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B235" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C235">
         <v>1</v>
@@ -7530,10 +7545,10 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B236" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C236">
         <v>1</v>
@@ -7544,10 +7559,10 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B237" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C237">
         <v>1</v>
@@ -7558,10 +7573,10 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B238" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C238">
         <v>1</v>
@@ -7572,10 +7587,10 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B239" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C239">
         <v>1</v>
@@ -7586,10 +7601,10 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B240" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C240">
         <v>1</v>
@@ -7600,10 +7615,10 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B241" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C241">
         <v>1</v>
@@ -7614,10 +7629,10 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B242" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C242">
         <v>1</v>
@@ -7637,10 +7652,10 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B243" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C243">
         <v>1</v>
@@ -7651,10 +7666,10 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B244" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C244">
         <v>1</v>
@@ -7665,10 +7680,10 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B245" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C245">
         <v>1</v>
@@ -7683,15 +7698,15 @@
         <v>20</v>
       </c>
       <c r="K245" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B246" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C246">
         <v>1</v>
@@ -7706,15 +7721,15 @@
         <v>24</v>
       </c>
       <c r="K246" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B247" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C247">
         <v>1</v>
@@ -7723,15 +7738,15 @@
         <v>0</v>
       </c>
       <c r="K247" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B248" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C248">
         <v>1</v>
@@ -7740,15 +7755,15 @@
         <v>0</v>
       </c>
       <c r="K248" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B249" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C249">
         <v>1</v>
@@ -7763,15 +7778,15 @@
         <v>143</v>
       </c>
       <c r="K249" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B250" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C250">
         <v>1</v>
@@ -7782,10 +7797,10 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B251" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C251">
         <v>1</v>
@@ -7797,18 +7812,18 @@
         <v>19</v>
       </c>
       <c r="F251" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="K251" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B252" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C252">
         <v>1</v>
@@ -7823,15 +7838,15 @@
         <v>33</v>
       </c>
       <c r="K252" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B253" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C253">
         <v>1</v>
@@ -7846,15 +7861,15 @@
         <v>359</v>
       </c>
       <c r="K253" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B254" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C254">
         <v>1</v>
@@ -7865,10 +7880,10 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B255" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C255">
         <v>1</v>
@@ -7879,10 +7894,10 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B256" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C256">
         <v>1</v>
@@ -7893,10 +7908,10 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B257" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C257">
         <v>1</v>
@@ -7907,10 +7922,10 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B258" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C258">
         <v>1</v>
@@ -7921,10 +7936,10 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B259" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C259">
         <v>1</v>
@@ -7935,10 +7950,10 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B260" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C260">
         <v>1</v>
@@ -7949,10 +7964,10 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B261" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C261">
         <v>1</v>
@@ -7963,10 +7978,10 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B262" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C262">
         <v>1</v>
@@ -7990,15 +8005,15 @@
         <v>15</v>
       </c>
       <c r="K262" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B263" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="C263">
         <v>1</v>
@@ -8009,10 +8024,10 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B264" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C264">
         <v>1</v>
@@ -8023,10 +8038,10 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B265" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C265">
         <v>1</v>
@@ -8037,10 +8052,10 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B266" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C266">
         <v>1</v>
@@ -8051,10 +8066,10 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B267" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C267">
         <v>1</v>
@@ -8065,10 +8080,10 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B268" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C268">
         <v>1</v>
@@ -8079,10 +8094,10 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B269" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C269">
         <v>1</v>
@@ -8097,15 +8112,15 @@
         <v>20</v>
       </c>
       <c r="K269" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B270" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C270">
         <v>1</v>
@@ -8116,10 +8131,10 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B271" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C271">
         <v>1</v>
@@ -8130,10 +8145,10 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B272" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C272">
         <v>1</v>
@@ -8144,10 +8159,10 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B273" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C273">
         <v>1</v>
@@ -8162,15 +8177,15 @@
         <v>24</v>
       </c>
       <c r="K273" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B274" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C274">
         <v>1</v>
@@ -8182,18 +8197,18 @@
         <v>19</v>
       </c>
       <c r="F274" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="K274" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B275" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C275">
         <v>1</v>
@@ -8204,24 +8219,24 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B276" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C276">
         <v>1</v>
       </c>
       <c r="D276">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B277" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C277">
         <v>1</v>
@@ -8232,10 +8247,10 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B278" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C278">
         <v>1</v>
@@ -8246,10 +8261,10 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B279" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C279">
         <v>1</v>
@@ -8261,18 +8276,18 @@
         <v>19</v>
       </c>
       <c r="F279" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="K279" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B280" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C280">
         <v>1</v>
@@ -8283,10 +8298,10 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B281" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C281">
         <v>1</v>
@@ -8297,10 +8312,10 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B282" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C282">
         <v>1</v>
@@ -8311,10 +8326,10 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B283" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C283">
         <v>1</v>
@@ -8325,10 +8340,10 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B284" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C284">
         <v>1</v>
@@ -8339,10 +8354,10 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B285" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C285">
         <v>1</v>
@@ -8353,10 +8368,10 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B286" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C286">
         <v>1</v>
@@ -8367,10 +8382,10 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B287" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C287">
         <v>1</v>
@@ -8381,10 +8396,10 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B288" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C288">
         <v>1</v>
@@ -8395,10 +8410,10 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B289" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C289">
         <v>1</v>
@@ -8409,10 +8424,10 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B290" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C290">
         <v>1</v>
@@ -8423,10 +8438,10 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B291" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C291">
         <v>1</v>
@@ -8437,10 +8452,10 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B292" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C292">
         <v>1</v>
@@ -8464,15 +8479,15 @@
         <v>15</v>
       </c>
       <c r="K292" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B293" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C293">
         <v>1</v>
@@ -8483,10 +8498,10 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B294" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="C294">
         <v>1</v>
@@ -8497,10 +8512,10 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B295" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C295">
         <v>1</v>
@@ -8511,10 +8526,10 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B296" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C296">
         <v>1</v>
@@ -8525,10 +8540,10 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B297" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C297">
         <v>1</v>
@@ -8539,10 +8554,10 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B298" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C298">
         <v>1</v>
@@ -8553,10 +8568,10 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B299" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C299">
         <v>1</v>
@@ -8580,15 +8595,15 @@
         <v>15</v>
       </c>
       <c r="K299" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B300" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C300">
         <v>1</v>
@@ -8599,10 +8614,10 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B301" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C301">
         <v>1</v>
@@ -8613,10 +8628,10 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B302" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="C302">
         <v>1</v>
@@ -8627,10 +8642,10 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B303" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="C303">
         <v>1</v>
@@ -8641,10 +8656,10 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B304" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C304">
         <v>1</v>
@@ -8655,10 +8670,10 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B305" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C305">
         <v>1</v>
@@ -8682,15 +8697,15 @@
         <v>15</v>
       </c>
       <c r="K305" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B306" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C306">
         <v>1</v>
@@ -8701,10 +8716,10 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B307" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C307">
         <v>1</v>
@@ -8715,10 +8730,10 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B308" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C308">
         <v>1</v>
@@ -8729,10 +8744,10 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="B309" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C309">
         <v>1</v>
@@ -8743,10 +8758,10 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="B310" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C310">
         <v>1</v>
@@ -8757,10 +8772,10 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B311" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C311">
         <v>1</v>
@@ -8771,10 +8786,10 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B312" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C312">
         <v>1</v>
@@ -8783,15 +8798,15 @@
         <v>0</v>
       </c>
       <c r="K312" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B313" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C313">
         <v>1</v>
@@ -8815,15 +8830,15 @@
         <v>15</v>
       </c>
       <c r="K313" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="B314" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C314">
         <v>1</v>
@@ -8838,15 +8853,15 @@
         <v>24</v>
       </c>
       <c r="K314" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B315" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C315">
         <v>1</v>
@@ -8857,10 +8872,10 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B316" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="C316">
         <v>1</v>
@@ -8871,10 +8886,10 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="B317" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C317">
         <v>1</v>
@@ -8885,10 +8900,10 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="B318" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C318">
         <v>1</v>
@@ -8899,10 +8914,10 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="B319" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C319">
         <v>1</v>
@@ -8917,15 +8932,15 @@
         <v>24</v>
       </c>
       <c r="K319" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B320" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C320">
         <v>1</v>
@@ -8936,10 +8951,10 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B321" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C321">
         <v>1</v>
@@ -8950,10 +8965,10 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="B322" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="C322">
         <v>1</v>
@@ -8964,10 +8979,10 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B323" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C323">
         <v>1</v>
@@ -8978,10 +8993,10 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B324" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C324">
         <v>1</v>
@@ -8996,15 +9011,15 @@
         <v>87</v>
       </c>
       <c r="K324" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B325" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C325">
         <v>1</v>
@@ -9015,10 +9030,10 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="B326" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="C326">
         <v>1</v>
@@ -9029,10 +9044,10 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B327" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C327">
         <v>1</v>
@@ -9043,10 +9058,10 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B328" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="C328">
         <v>1</v>
@@ -9055,15 +9070,15 @@
         <v>0</v>
       </c>
       <c r="K328" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B329" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C329">
         <v>1</v>
@@ -9074,10 +9089,10 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B330" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="C330">
         <v>1</v>
@@ -9088,10 +9103,10 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B331" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="C331">
         <v>1</v>
@@ -9102,10 +9117,10 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="B332" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="C332">
         <v>1</v>
@@ -9116,10 +9131,10 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B333" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C333">
         <v>1</v>
@@ -9130,10 +9145,10 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B334" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="C334">
         <v>1</v>
@@ -9144,10 +9159,10 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="B335" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="C335">
         <v>1</v>
@@ -9158,10 +9173,10 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B336" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C336">
         <v>1</v>
@@ -9172,10 +9187,10 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="B337" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="C337">
         <v>1</v>
@@ -9186,10 +9201,10 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B338" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="C338">
         <v>1</v>
@@ -9200,10 +9215,10 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="B339" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C339">
         <v>1</v>
@@ -9214,10 +9229,10 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B340" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C340">
         <v>1</v>
@@ -9228,10 +9243,10 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B341" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C341">
         <v>1</v>
@@ -9255,15 +9270,15 @@
         <v>29</v>
       </c>
       <c r="K341" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B342" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C342">
         <v>1</v>
@@ -9275,18 +9290,18 @@
         <v>19</v>
       </c>
       <c r="F342" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="K342" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B343" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C343">
         <v>1</v>
@@ -9297,10 +9312,10 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B344" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C344">
         <v>1</v>
@@ -9312,18 +9327,18 @@
         <v>19</v>
       </c>
       <c r="F344" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="K344" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B345" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C345">
         <v>1</v>
@@ -9334,10 +9349,10 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B346" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C346">
         <v>1</v>
@@ -9348,10 +9363,10 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B347" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C347">
         <v>1</v>
@@ -9362,10 +9377,10 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B348" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C348">
         <v>1</v>
@@ -9376,10 +9391,10 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B349" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C349">
         <v>1</v>
@@ -9390,10 +9405,10 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B350" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="C350">
         <v>1</v>
@@ -9404,10 +9419,10 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B351" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C351">
         <v>1</v>
@@ -9418,10 +9433,10 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B352" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C352">
         <v>1</v>
@@ -9432,10 +9447,10 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B353" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C353">
         <v>1</v>
@@ -9446,10 +9461,10 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B354" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C354">
         <v>1</v>
@@ -9460,10 +9475,10 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="B355" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C355">
         <v>1</v>
@@ -9474,10 +9489,10 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B356" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="C356">
         <v>1</v>
@@ -9488,16 +9503,16 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B357" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C357">
         <v>1</v>
       </c>
       <c r="D357">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E357" t="s">
         <v>13</v>
@@ -9515,15 +9530,15 @@
         <v>15</v>
       </c>
       <c r="K357" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B358" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C358">
         <v>1</v>
@@ -9534,10 +9549,10 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B359" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C359">
         <v>1</v>
@@ -9548,10 +9563,10 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B360" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C360">
         <v>1</v>
@@ -9562,10 +9577,10 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B361" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C361">
         <v>1</v>
@@ -9576,24 +9591,24 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B362" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="C362">
         <v>1</v>
       </c>
       <c r="D362">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B363" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="C363">
         <v>1</v>
@@ -9604,10 +9619,10 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B364" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="C364">
         <v>1</v>
@@ -9625,18 +9640,33 @@
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C2" t="s">
+        <v>445</v>
+      </c>
+      <c r="D2" t="s">
+        <v>902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Map: WP-B1 Arthas Moloch — Chart-Welt „Moloch“ an arthas_moloch gelinkt + Opt-in-Name-Override im Welten-Sheet (Session 254) (#285)
- map-worlds-core: Welten-Sheet-Spalte Name-Override (display-only; Welt-ID, Matching und Kurations-Ziele bleiben auf dem Excel-Namen), locationId-Override tri-state (leer = nicht angefasst), Legacy-3-Spalten-Header wird weiter gelesen
- import-map-worlds: --sync-curation schreibt das 4-Spalten-Layout; Name-only-Zeilen behalten leere locationId-Zelle
- Kurations-Excel: arthas_moloch → link/moloch (Kuration) + moloch → „Arthas Moloch“ (Welten); per Freigabe eingetragen, via --sync-curation normalisiert
- map-worlds.json/review regeneriert: moloch = Arthas Moloch mit 2 Werken; Abdeckung 1354/1710 (79.2 %), Worklist 237
- test-map-worlds: 47/47 grün (neue Override-Fälle inkl. WP-B1-Szenario); Fahrplan-Haken ✔ 254 + Impl-Report
</commit_message>
<xml_diff>
--- a/scripts/seed-data/source/map-worlds-curation.xlsx
+++ b/scripts/seed-data/source/map-worlds-curation.xlsx
@@ -1355,6 +1355,9 @@
     <t>Arthas Moloch</t>
   </si>
   <si>
+    <t>moloch</t>
+  </si>
+  <si>
     <t>arx_tyrannus</t>
   </si>
   <si>
@@ -2715,6 +2718,12 @@
   </si>
   <si>
     <t>locationId-Override</t>
+  </si>
+  <si>
+    <t>Name-Override</t>
+  </si>
+  <si>
+    <t>WP-B1: Chart-Welt „Moloch“ = Arthas Moloch (nicht Moloch III / Molech)</t>
   </si>
 </sst>
 </file>
@@ -2852,7 +2861,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>19</v>
@@ -6272,15 +6281,21 @@
         <v>1</v>
       </c>
       <c r="D162">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E162" t="s">
+        <v>57</v>
+      </c>
+      <c r="F162" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B163" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C163">
         <v>1</v>
@@ -6292,18 +6307,18 @@
         <v>19</v>
       </c>
       <c r="F163" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K163" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B164" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C164">
         <v>1</v>
@@ -6314,10 +6329,10 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B165" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C165">
         <v>1</v>
@@ -6328,10 +6343,10 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B166" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C166">
         <v>1</v>
@@ -6342,10 +6357,10 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B167" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C167">
         <v>1</v>
@@ -6356,10 +6371,10 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B168" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C168">
         <v>1</v>
@@ -6370,10 +6385,10 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B169" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C169">
         <v>1</v>
@@ -6384,10 +6399,10 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B170" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C170">
         <v>1</v>
@@ -6398,10 +6413,10 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B171" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C171">
         <v>1</v>
@@ -6412,10 +6427,10 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B172" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C172">
         <v>1</v>
@@ -6426,24 +6441,24 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B173" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C173">
         <v>1</v>
       </c>
       <c r="D173">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B174" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C174">
         <v>1</v>
@@ -6467,15 +6482,15 @@
         <v>29</v>
       </c>
       <c r="K174" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B175" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C175">
         <v>1</v>
@@ -6499,15 +6514,15 @@
         <v>15</v>
       </c>
       <c r="K175" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B176" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C176">
         <v>1</v>
@@ -6518,10 +6533,10 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B177" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -6530,15 +6545,15 @@
         <v>0</v>
       </c>
       <c r="K177" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B178" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C178">
         <v>1</v>
@@ -6549,10 +6564,10 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B179" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -6563,10 +6578,10 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B180" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C180">
         <v>1</v>
@@ -6577,10 +6592,10 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B181" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C181">
         <v>1</v>
@@ -6591,10 +6606,10 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B182" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C182">
         <v>1</v>
@@ -6605,10 +6620,10 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B183" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C183">
         <v>1</v>
@@ -6620,18 +6635,18 @@
         <v>19</v>
       </c>
       <c r="F183" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K183" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B184" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C184">
         <v>1</v>
@@ -6642,10 +6657,10 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B185" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C185">
         <v>1</v>
@@ -6656,10 +6671,10 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B186" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C186">
         <v>1</v>
@@ -6670,10 +6685,10 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B187" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C187">
         <v>1</v>
@@ -6684,10 +6699,10 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B188" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C188">
         <v>1</v>
@@ -6711,15 +6726,15 @@
         <v>15</v>
       </c>
       <c r="K188" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B189" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C189">
         <v>1</v>
@@ -6730,10 +6745,10 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B190" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C190">
         <v>1</v>
@@ -6744,10 +6759,10 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B191" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C191">
         <v>1</v>
@@ -6762,15 +6777,15 @@
         <v>24</v>
       </c>
       <c r="K191" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B192" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C192">
         <v>1</v>
@@ -6781,10 +6796,10 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B193" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C193">
         <v>1</v>
@@ -6795,10 +6810,10 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B194" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C194">
         <v>1</v>
@@ -6809,10 +6824,10 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B195" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C195">
         <v>1</v>
@@ -6823,10 +6838,10 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B196" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C196">
         <v>1</v>
@@ -6837,10 +6852,10 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B197" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C197">
         <v>1</v>
@@ -6851,10 +6866,10 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B198" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C198">
         <v>1</v>
@@ -6865,10 +6880,10 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B199" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C199">
         <v>1</v>
@@ -6879,10 +6894,10 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B200" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C200">
         <v>1</v>
@@ -6893,10 +6908,10 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B201" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C201">
         <v>1</v>
@@ -6907,10 +6922,10 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B202" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C202">
         <v>1</v>
@@ -6921,10 +6936,10 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B203" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C203">
         <v>1</v>
@@ -6948,15 +6963,15 @@
         <v>15</v>
       </c>
       <c r="K203" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B204" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C204">
         <v>1</v>
@@ -6967,10 +6982,10 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B205" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C205">
         <v>1</v>
@@ -6994,15 +7009,15 @@
         <v>15</v>
       </c>
       <c r="K205" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B206" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C206">
         <v>1</v>
@@ -7026,15 +7041,15 @@
         <v>29</v>
       </c>
       <c r="K206" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B207" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C207">
         <v>1</v>
@@ -7045,10 +7060,10 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B208" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C208">
         <v>1</v>
@@ -7057,15 +7072,15 @@
         <v>0</v>
       </c>
       <c r="K208" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B209" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C209">
         <v>1</v>
@@ -7080,15 +7095,15 @@
         <v>24</v>
       </c>
       <c r="K209" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B210" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C210">
         <v>1</v>
@@ -7099,10 +7114,10 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B211" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C211">
         <v>1</v>
@@ -7113,10 +7128,10 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B212" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C212">
         <v>1</v>
@@ -7131,15 +7146,15 @@
         <v>33</v>
       </c>
       <c r="K212" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B213" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C213">
         <v>1</v>
@@ -7150,10 +7165,10 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B214" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C214">
         <v>1</v>
@@ -7164,10 +7179,10 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B215" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C215">
         <v>1</v>
@@ -7178,10 +7193,10 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B216" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C216">
         <v>1</v>
@@ -7192,10 +7207,10 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B217" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C217">
         <v>1</v>
@@ -7206,10 +7221,10 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B218" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C218">
         <v>1</v>
@@ -7220,24 +7235,24 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B219" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C219">
         <v>1</v>
       </c>
       <c r="D219">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B220" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C220">
         <v>1</v>
@@ -7248,10 +7263,10 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B221" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C221">
         <v>1</v>
@@ -7262,10 +7277,10 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B222" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C222">
         <v>1</v>
@@ -7276,10 +7291,10 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B223" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C223">
         <v>1</v>
@@ -7290,10 +7305,10 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B224" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C224">
         <v>1</v>
@@ -7304,10 +7319,10 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B225" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C225">
         <v>1</v>
@@ -7318,10 +7333,10 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B226" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C226">
         <v>1</v>
@@ -7345,15 +7360,15 @@
         <v>15</v>
       </c>
       <c r="K226" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B227" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C227">
         <v>1</v>
@@ -7368,15 +7383,15 @@
         <v>24</v>
       </c>
       <c r="K227" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B228" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C228">
         <v>1</v>
@@ -7387,10 +7402,10 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B229" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C229">
         <v>1</v>
@@ -7414,15 +7429,15 @@
         <v>15</v>
       </c>
       <c r="K229" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B230" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C230">
         <v>1</v>
@@ -7433,10 +7448,10 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B231" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C231">
         <v>1</v>
@@ -7456,16 +7471,16 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B232" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C232">
         <v>1</v>
       </c>
       <c r="D232">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E232" t="s">
         <v>13</v>
@@ -7483,15 +7498,15 @@
         <v>29</v>
       </c>
       <c r="K232" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B233" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C233">
         <v>1</v>
@@ -7502,10 +7517,10 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B234" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C234">
         <v>1</v>
@@ -7516,10 +7531,10 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B235" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C235">
         <v>1</v>
@@ -7530,10 +7545,10 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B236" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C236">
         <v>1</v>
@@ -7544,10 +7559,10 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B237" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C237">
         <v>1</v>
@@ -7558,10 +7573,10 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B238" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C238">
         <v>1</v>
@@ -7572,10 +7587,10 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B239" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C239">
         <v>1</v>
@@ -7586,10 +7601,10 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B240" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C240">
         <v>1</v>
@@ -7600,10 +7615,10 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B241" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C241">
         <v>1</v>
@@ -7614,10 +7629,10 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B242" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C242">
         <v>1</v>
@@ -7637,10 +7652,10 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B243" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C243">
         <v>1</v>
@@ -7651,10 +7666,10 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B244" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C244">
         <v>1</v>
@@ -7665,10 +7680,10 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B245" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C245">
         <v>1</v>
@@ -7683,15 +7698,15 @@
         <v>20</v>
       </c>
       <c r="K245" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B246" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C246">
         <v>1</v>
@@ -7706,15 +7721,15 @@
         <v>24</v>
       </c>
       <c r="K246" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B247" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C247">
         <v>1</v>
@@ -7723,15 +7738,15 @@
         <v>0</v>
       </c>
       <c r="K247" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B248" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C248">
         <v>1</v>
@@ -7740,15 +7755,15 @@
         <v>0</v>
       </c>
       <c r="K248" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B249" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C249">
         <v>1</v>
@@ -7763,15 +7778,15 @@
         <v>143</v>
       </c>
       <c r="K249" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B250" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C250">
         <v>1</v>
@@ -7782,10 +7797,10 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B251" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C251">
         <v>1</v>
@@ -7797,18 +7812,18 @@
         <v>19</v>
       </c>
       <c r="F251" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="K251" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B252" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C252">
         <v>1</v>
@@ -7823,15 +7838,15 @@
         <v>33</v>
       </c>
       <c r="K252" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B253" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C253">
         <v>1</v>
@@ -7846,15 +7861,15 @@
         <v>359</v>
       </c>
       <c r="K253" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B254" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C254">
         <v>1</v>
@@ -7865,10 +7880,10 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B255" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C255">
         <v>1</v>
@@ -7879,10 +7894,10 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B256" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C256">
         <v>1</v>
@@ -7893,10 +7908,10 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B257" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C257">
         <v>1</v>
@@ -7907,10 +7922,10 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B258" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C258">
         <v>1</v>
@@ -7921,10 +7936,10 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B259" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C259">
         <v>1</v>
@@ -7935,10 +7950,10 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B260" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C260">
         <v>1</v>
@@ -7949,10 +7964,10 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B261" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C261">
         <v>1</v>
@@ -7963,10 +7978,10 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B262" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C262">
         <v>1</v>
@@ -7990,15 +8005,15 @@
         <v>15</v>
       </c>
       <c r="K262" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B263" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="C263">
         <v>1</v>
@@ -8009,10 +8024,10 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B264" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C264">
         <v>1</v>
@@ -8023,10 +8038,10 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B265" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C265">
         <v>1</v>
@@ -8037,10 +8052,10 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B266" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C266">
         <v>1</v>
@@ -8051,10 +8066,10 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B267" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C267">
         <v>1</v>
@@ -8065,10 +8080,10 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B268" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C268">
         <v>1</v>
@@ -8079,10 +8094,10 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B269" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C269">
         <v>1</v>
@@ -8097,15 +8112,15 @@
         <v>20</v>
       </c>
       <c r="K269" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B270" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C270">
         <v>1</v>
@@ -8116,10 +8131,10 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B271" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C271">
         <v>1</v>
@@ -8130,10 +8145,10 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B272" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C272">
         <v>1</v>
@@ -8144,10 +8159,10 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B273" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C273">
         <v>1</v>
@@ -8162,15 +8177,15 @@
         <v>24</v>
       </c>
       <c r="K273" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B274" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C274">
         <v>1</v>
@@ -8182,18 +8197,18 @@
         <v>19</v>
       </c>
       <c r="F274" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="K274" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B275" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C275">
         <v>1</v>
@@ -8204,24 +8219,24 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B276" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C276">
         <v>1</v>
       </c>
       <c r="D276">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B277" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C277">
         <v>1</v>
@@ -8232,10 +8247,10 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B278" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C278">
         <v>1</v>
@@ -8246,10 +8261,10 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B279" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C279">
         <v>1</v>
@@ -8261,18 +8276,18 @@
         <v>19</v>
       </c>
       <c r="F279" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="K279" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B280" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C280">
         <v>1</v>
@@ -8283,10 +8298,10 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B281" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C281">
         <v>1</v>
@@ -8297,10 +8312,10 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B282" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C282">
         <v>1</v>
@@ -8311,10 +8326,10 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B283" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C283">
         <v>1</v>
@@ -8325,10 +8340,10 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B284" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C284">
         <v>1</v>
@@ -8339,10 +8354,10 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B285" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C285">
         <v>1</v>
@@ -8353,10 +8368,10 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B286" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C286">
         <v>1</v>
@@ -8367,10 +8382,10 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B287" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C287">
         <v>1</v>
@@ -8381,10 +8396,10 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B288" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C288">
         <v>1</v>
@@ -8395,10 +8410,10 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B289" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C289">
         <v>1</v>
@@ -8409,10 +8424,10 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B290" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C290">
         <v>1</v>
@@ -8423,10 +8438,10 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B291" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C291">
         <v>1</v>
@@ -8437,10 +8452,10 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B292" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C292">
         <v>1</v>
@@ -8464,15 +8479,15 @@
         <v>15</v>
       </c>
       <c r="K292" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B293" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C293">
         <v>1</v>
@@ -8483,10 +8498,10 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B294" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="C294">
         <v>1</v>
@@ -8497,10 +8512,10 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B295" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C295">
         <v>1</v>
@@ -8511,10 +8526,10 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B296" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C296">
         <v>1</v>
@@ -8525,10 +8540,10 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B297" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C297">
         <v>1</v>
@@ -8539,10 +8554,10 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B298" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C298">
         <v>1</v>
@@ -8553,10 +8568,10 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B299" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C299">
         <v>1</v>
@@ -8580,15 +8595,15 @@
         <v>15</v>
       </c>
       <c r="K299" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B300" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C300">
         <v>1</v>
@@ -8599,10 +8614,10 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B301" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C301">
         <v>1</v>
@@ -8613,10 +8628,10 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B302" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="C302">
         <v>1</v>
@@ -8627,10 +8642,10 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B303" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="C303">
         <v>1</v>
@@ -8641,10 +8656,10 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B304" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C304">
         <v>1</v>
@@ -8655,10 +8670,10 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B305" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C305">
         <v>1</v>
@@ -8682,15 +8697,15 @@
         <v>15</v>
       </c>
       <c r="K305" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B306" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C306">
         <v>1</v>
@@ -8701,10 +8716,10 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B307" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C307">
         <v>1</v>
@@ -8715,10 +8730,10 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B308" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C308">
         <v>1</v>
@@ -8729,10 +8744,10 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="B309" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C309">
         <v>1</v>
@@ -8743,10 +8758,10 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="B310" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C310">
         <v>1</v>
@@ -8757,10 +8772,10 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B311" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C311">
         <v>1</v>
@@ -8771,10 +8786,10 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B312" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C312">
         <v>1</v>
@@ -8783,15 +8798,15 @@
         <v>0</v>
       </c>
       <c r="K312" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B313" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C313">
         <v>1</v>
@@ -8815,15 +8830,15 @@
         <v>15</v>
       </c>
       <c r="K313" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="B314" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C314">
         <v>1</v>
@@ -8838,15 +8853,15 @@
         <v>24</v>
       </c>
       <c r="K314" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B315" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C315">
         <v>1</v>
@@ -8857,10 +8872,10 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B316" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="C316">
         <v>1</v>
@@ -8871,10 +8886,10 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="B317" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C317">
         <v>1</v>
@@ -8885,10 +8900,10 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="B318" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C318">
         <v>1</v>
@@ -8899,10 +8914,10 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="B319" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C319">
         <v>1</v>
@@ -8917,15 +8932,15 @@
         <v>24</v>
       </c>
       <c r="K319" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B320" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C320">
         <v>1</v>
@@ -8936,10 +8951,10 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B321" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C321">
         <v>1</v>
@@ -8950,10 +8965,10 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="B322" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="C322">
         <v>1</v>
@@ -8964,10 +8979,10 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B323" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C323">
         <v>1</v>
@@ -8978,10 +8993,10 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B324" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C324">
         <v>1</v>
@@ -8996,15 +9011,15 @@
         <v>87</v>
       </c>
       <c r="K324" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B325" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C325">
         <v>1</v>
@@ -9015,10 +9030,10 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="B326" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="C326">
         <v>1</v>
@@ -9029,10 +9044,10 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B327" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C327">
         <v>1</v>
@@ -9043,10 +9058,10 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B328" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="C328">
         <v>1</v>
@@ -9055,15 +9070,15 @@
         <v>0</v>
       </c>
       <c r="K328" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B329" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C329">
         <v>1</v>
@@ -9074,10 +9089,10 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B330" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="C330">
         <v>1</v>
@@ -9088,10 +9103,10 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B331" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="C331">
         <v>1</v>
@@ -9102,10 +9117,10 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="B332" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="C332">
         <v>1</v>
@@ -9116,10 +9131,10 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B333" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C333">
         <v>1</v>
@@ -9130,10 +9145,10 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B334" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="C334">
         <v>1</v>
@@ -9144,10 +9159,10 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="B335" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="C335">
         <v>1</v>
@@ -9158,10 +9173,10 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B336" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C336">
         <v>1</v>
@@ -9172,10 +9187,10 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="B337" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="C337">
         <v>1</v>
@@ -9186,10 +9201,10 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B338" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="C338">
         <v>1</v>
@@ -9200,10 +9215,10 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="B339" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C339">
         <v>1</v>
@@ -9214,10 +9229,10 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B340" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C340">
         <v>1</v>
@@ -9228,10 +9243,10 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B341" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C341">
         <v>1</v>
@@ -9255,15 +9270,15 @@
         <v>29</v>
       </c>
       <c r="K341" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B342" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C342">
         <v>1</v>
@@ -9275,18 +9290,18 @@
         <v>19</v>
       </c>
       <c r="F342" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="K342" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B343" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C343">
         <v>1</v>
@@ -9297,10 +9312,10 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B344" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C344">
         <v>1</v>
@@ -9312,18 +9327,18 @@
         <v>19</v>
       </c>
       <c r="F344" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="K344" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B345" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C345">
         <v>1</v>
@@ -9334,10 +9349,10 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B346" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C346">
         <v>1</v>
@@ -9348,10 +9363,10 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B347" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C347">
         <v>1</v>
@@ -9362,10 +9377,10 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B348" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C348">
         <v>1</v>
@@ -9376,10 +9391,10 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B349" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C349">
         <v>1</v>
@@ -9390,10 +9405,10 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B350" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="C350">
         <v>1</v>
@@ -9404,10 +9419,10 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B351" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C351">
         <v>1</v>
@@ -9418,10 +9433,10 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B352" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C352">
         <v>1</v>
@@ -9432,10 +9447,10 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B353" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C353">
         <v>1</v>
@@ -9446,10 +9461,10 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B354" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C354">
         <v>1</v>
@@ -9460,10 +9475,10 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="B355" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C355">
         <v>1</v>
@@ -9474,10 +9489,10 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B356" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="C356">
         <v>1</v>
@@ -9488,16 +9503,16 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B357" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C357">
         <v>1</v>
       </c>
       <c r="D357">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E357" t="s">
         <v>13</v>
@@ -9515,15 +9530,15 @@
         <v>15</v>
       </c>
       <c r="K357" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B358" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C358">
         <v>1</v>
@@ -9534,10 +9549,10 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B359" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C359">
         <v>1</v>
@@ -9548,10 +9563,10 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B360" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C360">
         <v>1</v>
@@ -9562,10 +9577,10 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B361" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C361">
         <v>1</v>
@@ -9576,24 +9591,24 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B362" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="C362">
         <v>1</v>
       </c>
       <c r="D362">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B363" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="C363">
         <v>1</v>
@@ -9604,10 +9619,10 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B364" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="C364">
         <v>1</v>
@@ -9625,18 +9640,33 @@
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C2" t="s">
+        <v>445</v>
+      </c>
+      <c r="D2" t="s">
+        <v>902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>